<commit_message>
MXSC task: fix change-point bugs and redesign for the 2026 cohort
The 2025 task code had two change-point bugs:
- the post-switch drift dropped the trial's sign, so after the switch
  the pigeon always drifted right (both LowHigh and HighLow);
- switch_time was an unrounded median RT, so an even-length fixed block
  could give a half-integer that never equals the integer step counter,
  and the switch never fired.

This version (used to collect the 2026 cohort, Aug-Sep 2026) re-applies
the sign at the switch, rounds switch_time and logs it per trial, and
removes the unused mixed-SNR block, so the change-point blocks are now
3/4 instead of 4/5. High SNR goes from 0.4 to 0.6 (tc_step_mean 0.02 ->
0.03); Test_cpDesign.ipynb is the design study behind that choice.

PigeonTask.psyexp is kept as PigeonTask_obsolete.psyexp: the JS was
edited directly and no longer compiles from it.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/task/MXSC/Resources/Pigeon_change_InstructionsConditions.xlsx
+++ b/task/MXSC/Resources/Pigeon_change_InstructionsConditions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10703"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ishankalburge/Documents/penn/pigeons-lohi-snr-v1/Resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jigold/Library/CloudStorage/Box-Box/GoldLab/Projects/2025_Pigeon/Code/task/MXSC/Resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{306FF71C-6456-4D42-896D-8B412FDF9D2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{285EAD81-7C9F-5C4F-8DCB-2FCBC8771393}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="760" windowWidth="24600" windowHeight="12840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="760" windowWidth="24580" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,47 +38,35 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
-    <t xml:space="preserve">ic_message_string</t>
-  </si>
-  <si>
-    <t xml:space="preserve">You are in the change block. In this block, Petey will start out foraging either at night or during the day (indicated by the initial icon in the top right of the screen).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Partway through the trial, the time of day will change. If Petey starts out foraging during the day, then there will be a change to nighttime at some point during the trial, and vice versa.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Petey will keep heading toward the same pile of seeds for the whole trial -- the change only affects how quickly and reliably he gets there, not which pile he is heading for.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">You will also see a countdown timer indicating when this change will occur within a trial.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">You may receive a cash bonus based on your final score for the block.</t>
+    <t>ic_message_string</t>
+  </si>
+  <si>
+    <t>You are in the change block. In this block, Petey will start out foraging either at night or during the day (indicated by the initial icon in the top right of the screen).</t>
+  </si>
+  <si>
+    <t>Partway through the trial, the time of day will change. If Petey starts out foraging during the day, then there will be a change to nighttime at some point during the trial, and vice versa.</t>
+  </si>
+  <si>
+    <t>Petey will keep heading toward the same pile of seeds for the whole trial -- the change only affects how quickly and reliably he gets there, not which pile he is heading for.</t>
+  </si>
+  <si>
+    <t>You will also see a countdown timer indicating when this change will occur within a trial.</t>
+  </si>
+  <si>
+    <t>You may receive a bonus payment based on your final score for the block.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -89,7 +77,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -97,34 +85,15 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1" readingOrder="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -438,45 +407,45 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:1" ht="80" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:1" ht="80" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:1">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:1" ht="80" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:1">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:1" ht="48" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:1">
-      <c r="A6" s="2" t="s">
+    <row r="6" spans="1:1" ht="32" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:1">
-      <c r="A7" s="2"/>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A7" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>